<commit_message>
chore: update schedules 2026-08-11
</commit_message>
<xml_diff>
--- a/output/one_schedules_latest.xlsx
+++ b/output/one_schedules_latest.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -528,12 +528,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>ONE MAGDALENA</t>
+          <t>CAPE ARTEMISIO</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>ONE MAGDALENA 2630W</t>
+          <t>CAPE ARTEMISIO FI631A</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -543,12 +543,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>48</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -558,7 +558,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-08-10 05:12 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -585,22 +585,22 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>SX1</t>
+          <t>JSM</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>CAPE ARTEMISIO</t>
+          <t>EMMANUEL P</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>CAPE ARTEMISIO FI631A</t>
+          <t>EMMANUEL P 012S</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -610,12 +610,12 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>54</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-08-10 05:12 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -652,22 +652,22 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>JSM</t>
+          <t>SX1</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>EMMANUEL P</t>
+          <t>SEASPAN BELIEF</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EMMANUEL P 012S</t>
+          <t>SEASPAN BELIEF 2632W</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -677,12 +677,12 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>56</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -692,7 +692,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-08-10 05:12 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -719,22 +719,22 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>SX1</t>
+          <t>JSM</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>SEASPAN BELIEF</t>
+          <t>NAVIOS CHRYSALIS</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>SEASPAN BELIEF 2632W</t>
+          <t>NAVIOS CHRYSALIS 016S</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -749,7 +749,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>55</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-08-10 05:12 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -786,22 +786,22 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>JSM</t>
+          <t>SX1</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>NAVIOS CHRYSALIS</t>
+          <t>MSC SHREYA B</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>NAVIOS CHRYSALIS 016S</t>
+          <t>MSC SHREYA B FI633A</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -811,12 +811,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>64</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -826,7 +826,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-08-10 05:12 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -858,17 +858,17 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>SX1</t>
+          <t>JSM</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>MSC SHREYA B</t>
+          <t>NAVIOS VERDE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>MSC SHREYA B FI633A</t>
+          <t>NAVIOS VERDE 186S</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-08-10 05:12 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -920,22 +920,22 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>JSM</t>
+          <t>SX1</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>NAVIOS VERDE</t>
+          <t>ESPIRITO SANTO EXPRESS</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>NAVIOS VERDE 186S</t>
+          <t>ESPIRITO SANTO EXPRESS 2634W</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -950,7 +950,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>55</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-08-10 05:12 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -992,17 +992,17 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>SX1</t>
+          <t>JSM</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>ESPIRITO SANTO EXPRESS</t>
+          <t>ATHENS BRIDGE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>ESPIRITO SANTO EXPRESS 2634W</t>
+          <t>ATHENS BRIDGE 1188S</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1027,14 +1027,14 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-08-10 05:12 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>HKHKG→SEGOT</t>
+          <t>HKHKG→NOOSL</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SEGOT</t>
+          <t>NOOSL</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1054,37 +1054,37 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>JSM</t>
+          <t>SX1</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>ATHENS BRIDGE</t>
+          <t>CAPE ARTEMISIO</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>ATHENS BRIDGE 1188S</t>
+          <t>CAPE ARTEMISIO FI631A</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>GOTHENBURG</t>
+          <t>ROTTERDAM</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>40</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-08-10 05:12 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1121,22 +1121,22 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>SX1</t>
+          <t>JSM</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>ONE MAGDALENA</t>
+          <t>EMMANUEL P</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>ONE MAGDALENA 2630W</t>
+          <t>EMMANUEL P 012S</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>46</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1188,22 +1188,22 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>SX1</t>
+          <t>JSM</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>CAPE ARTEMISIO</t>
+          <t>EMMANUEL P</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>CAPE ARTEMISIO FI631A</t>
+          <t>EMMANUEL P 012S</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1213,12 +1213,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>48</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1255,22 +1255,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>JSM</t>
+          <t>SX1</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>EMMANUEL P</t>
+          <t>SEASPAN BELIEF</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>EMMANUEL P 012S</t>
+          <t>SEASPAN BELIEF 2632W</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1280,12 +1280,12 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>48</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1332,12 +1332,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>EMMANUEL P</t>
+          <t>NAVIOS CHRYSALIS</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>EMMANUEL P 012S</t>
+          <t>NAVIOS CHRYSALIS 016S</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1347,12 +1347,12 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>47</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1389,22 +1389,22 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>SX1</t>
+          <t>JSM</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>SEASPAN BELIEF</t>
+          <t>NAVIOS CHRYSALIS</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>SEASPAN BELIEF 2632W</t>
+          <t>NAVIOS CHRYSALIS 016S</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1414,12 +1414,12 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>49</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1456,22 +1456,22 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>JSM</t>
+          <t>SX1</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>NAVIOS CHRYSALIS</t>
+          <t>MSC SHREYA B</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>NAVIOS CHRYSALIS 016S</t>
+          <t>MSC SHREYA B FI633A</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1481,12 +1481,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>56</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1496,7 +1496,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1523,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1533,12 +1533,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>NAVIOS CHRYSALIS</t>
+          <t>NAVIOS VERDE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>NAVIOS CHRYSALIS 016S</t>
+          <t>NAVIOS VERDE 186S</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1595,17 +1595,17 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>SX1</t>
+          <t>JSM</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>MSC SHREYA B</t>
+          <t>NAVIOS VERDE</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>MSC SHREYA B FI633A</t>
+          <t>NAVIOS VERDE 186S</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1657,22 +1657,22 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>JSM</t>
+          <t>SX1</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>NAVIOS VERDE</t>
+          <t>ESPIRITO SANTO EXPRESS</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>NAVIOS VERDE 186S</t>
+          <t>ESPIRITO SANTO EXPRESS 2634W</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1682,12 +1682,12 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>47</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1734,12 +1734,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>NAVIOS VERDE</t>
+          <t>ATHENS BRIDGE</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>NAVIOS VERDE 186S</t>
+          <t>ATHENS BRIDGE 1188S</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>47</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1796,17 +1796,17 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>SX1</t>
+          <t>JSM</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>ESPIRITO SANTO EXPRESS</t>
+          <t>ATHENS BRIDGE</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>ESPIRITO SANTO EXPRESS 2634W</t>
+          <t>ATHENS BRIDGE 1188S</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1816,12 +1816,12 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>49</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1831,49 +1831,45 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>HKHKG→NOOSL</t>
+          <t>VNSGN→NOTAE</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>NOOSL</t>
+          <t>NOTAE</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>HONG KONG</t>
+          <t>CAI MEP</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>JSM</t>
-        </is>
-      </c>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>ATHENS BRIDGE</t>
+          <t>TAN CANG CAI MEP INTERNATIONAL TERMINALCO.,LTD (WATER)</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>ATHENS BRIDGE 1188S</t>
+          <t>TAN CANG CAI MEP INTERNATIONAL TERMINALCO.,LTD (WATER)</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1883,12 +1879,12 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>40</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -1898,49 +1894,45 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>HKHKG→NOOSL</t>
+          <t>VNSGN→NOTAE</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>NOOSL</t>
+          <t>NOTAE</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>HONG KONG</t>
+          <t>CAI MEP</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>JSM</t>
-        </is>
-      </c>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>ATHENS BRIDGE</t>
+          <t>TAN CANG CAI MEP INTERNATIONAL TERMINALCO.,LTD (WATER)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>ATHENS BRIDGE 1188S</t>
+          <t>TAN CANG CAI MEP INTERNATIONAL TERMINALCO.,LTD (WATER)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1950,12 +1942,12 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>41</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -1965,7 +1957,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1992,7 +1984,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
@@ -2013,22 +2005,22 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>48</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>TRANSSHIPMENT (2)</t>
+          <t>TRANSSHIPMENT (3)</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2047,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
@@ -2076,22 +2068,22 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>57</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>TRANSSHIPMENT (2)</t>
+          <t>TRANSSHIPMENT (3)</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2110,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
@@ -2144,17 +2136,17 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>42</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>TRANSSHIPMENT (3)</t>
+          <t>TRANSSHIPMENT (2)</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2181,7 +2173,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
@@ -2207,7 +2199,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>48</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2217,7 +2209,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2244,7 +2236,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -2265,85 +2257,89 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>45</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>TRANSSHIPMENT (2)</t>
+          <t>TRANSSHIPMENT (3)</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:52 UTC</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>VNSGN→NOTAE</t>
+          <t>CNTAO→ITSPE</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>CNTAO</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>NOTAE</t>
+          <t>ITSPE</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>CAI MEP</t>
+          <t>QINGDAO, SHANDONG</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>PN3</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>TAN CANG CAI MEP INTERNATIONAL TERMINALCO.,LTD (WATER)</t>
+          <t>YM MOBILITY</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>TAN CANG CAI MEP INTERNATIONAL TERMINALCO.,LTD (WATER)</t>
+          <t>YM MOBILITY 090E</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>ROTTERDAM</t>
+          <t>LA SPEZIA</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>71</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>TRANSSHIPMENT (3)</t>
+          <t>TRANSSHIPMENT (1)</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2366,22 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>PN3</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>YM MOBILITY</t>
+          <t>ONE FUTURE</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>YM MOBILITY 090E</t>
+          <t>ONE FUTURE 009W</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2395,12 +2391,12 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>57</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -2410,7 +2406,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2462,12 +2458,12 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>67</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -2477,7 +2473,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2504,22 +2500,22 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>AX3</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>ONE FUTURE</t>
+          <t>TENO</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>ONE FUTURE 009W</t>
+          <t>TENO 2631E</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2529,12 +2525,12 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-11-05</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>80</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -2544,7 +2540,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2571,22 +2567,22 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>AX3</t>
+          <t>PN3</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>TENO</t>
+          <t>HYUNDAI FORWARD</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>TENO 2631E</t>
+          <t>HYUNDAI FORWARD 171E</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2601,7 +2597,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>79</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -2611,7 +2607,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2638,7 +2634,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2648,12 +2644,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>HYUNDAI FORWARD</t>
+          <t>ONE MODERN</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>HYUNDAI FORWARD 171E</t>
+          <t>ONE MODERN 082E</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2668,7 +2664,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>77</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -2678,7 +2674,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2705,22 +2701,22 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>PN3</t>
+          <t>AX3</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>ONE MODERN</t>
+          <t>SEASPAN ZAMBEZI</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>ONE MODERN 082E</t>
+          <t>SEASPAN ZAMBEZI 2632E</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2735,7 +2731,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>76</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -2745,7 +2741,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2772,22 +2768,22 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>AX3</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>SEASPAN ZAMBEZI</t>
+          <t>HMM LE HAVRE</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>SEASPAN ZAMBEZI 2632E</t>
+          <t>HMM LE HAVRE 019W</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2797,12 +2793,12 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-11-05</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>57</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -2812,7 +2808,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2864,12 +2860,12 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>60</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -2879,7 +2875,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2906,22 +2902,22 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>AX3</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>HMM LE HAVRE</t>
+          <t>POSORJA EXPRESS</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>HMM LE HAVRE 019W</t>
+          <t>POSORJA EXPRESS 2633E</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2931,12 +2927,12 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-11-05</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>72</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -2946,7 +2942,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2973,22 +2969,22 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>AX3</t>
+          <t>AX4</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>POSORJA EXPRESS</t>
+          <t>ONE COMPETENCE</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>POSORJA EXPRESS 2633E</t>
+          <t>ONE COMPETENCE 099E</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -3003,7 +2999,7 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>71</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -3013,7 +3009,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:53 UTC</t>
         </is>
       </c>
     </row>
@@ -3040,22 +3036,22 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>AX4</t>
+          <t>PN3</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>ONE COMPETENCE</t>
+          <t>HMM VANCOUVER</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>ONE COMPETENCE 099E</t>
+          <t>HMM VANCOUVER 307E</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3065,12 +3061,12 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-11-05</t>
+          <t>2026-11-12</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>76</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -3080,7 +3076,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:53 UTC</t>
         </is>
       </c>
     </row>
@@ -3107,22 +3103,22 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>PN3</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>HMM VANCOUVER</t>
+          <t>ONE FOREVER</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>HMM VANCOUVER 307E</t>
+          <t>ONE FOREVER 010W</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3132,12 +3128,12 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-11-12</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>57</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -3147,7 +3143,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:53 UTC</t>
         </is>
       </c>
     </row>
@@ -3199,12 +3195,12 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-11-05</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>67</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -3214,7 +3210,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:53 UTC</t>
         </is>
       </c>
     </row>
@@ -3241,22 +3237,22 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>PN3</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>ONE FOREVER</t>
+          <t>HYUNDAI SUPREME</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>ONE FOREVER 010W</t>
+          <t>HYUNDAI SUPREME 159E</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3266,12 +3262,12 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-11-05</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>79</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
@@ -3281,7 +3277,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:53 UTC</t>
         </is>
       </c>
     </row>
@@ -3308,22 +3304,22 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>PN3</t>
+          <t>AX4</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>HYUNDAI SUPREME</t>
+          <t>CONTI CONTESSA</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>HYUNDAI SUPREME 159E</t>
+          <t>CONTI CONTESSA 026E</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3333,12 +3329,12 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-11-12</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>71</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -3348,7 +3344,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:53 UTC</t>
         </is>
       </c>
     </row>
@@ -3375,22 +3371,22 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>AX4</t>
+          <t>AX3</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>CONTI CONTESSA</t>
+          <t>YOKOHAMA EXPRESS</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>CONTI CONTESSA 026E</t>
+          <t>YOKOHAMA EXPRESS 2634E</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3405,7 +3401,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>70</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
@@ -3415,7 +3411,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:53 UTC</t>
         </is>
       </c>
     </row>
@@ -3442,22 +3438,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>AX3</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>YOKOHAMA EXPRESS</t>
+          <t>HMM COPENHAGEN</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>YOKOHAMA EXPRESS 2634E</t>
+          <t>HMM COPENHAGEN 020W</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3467,12 +3463,12 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-11-12</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>50</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -3482,7 +3478,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:53 UTC</t>
         </is>
       </c>
     </row>
@@ -3534,12 +3530,12 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-11-02</t>
+          <t>2026-11-05</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>60</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -3549,7 +3545,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:53 UTC</t>
         </is>
       </c>
     </row>
@@ -3576,22 +3572,22 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>AX4</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>HMM COPENHAGEN</t>
+          <t>HYUNDAI COURAGE</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>HMM COPENHAGEN 020W</t>
+          <t>HYUNDAI COURAGE 125E</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3601,12 +3597,12 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-11-05</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>72</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
@@ -3616,7 +3612,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>2026-08-10 05:13 UTC</t>
+          <t>2026-08-11 04:53 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>